<commit_message>
Stable and Recovery Point
</commit_message>
<xml_diff>
--- a/Aivellum_Sales.xlsx
+++ b/Aivellum_Sales.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="314">
   <si>
     <t>S.NO</t>
   </si>
@@ -112,6 +112,15 @@
     <t>2025-12-16</t>
   </si>
   <si>
+    <t>2025-12-17</t>
+  </si>
+  <si>
+    <t>2025-12-20</t>
+  </si>
+  <si>
+    <t>2025-12-19</t>
+  </si>
+  <si>
     <t>00:33:28 UTC</t>
   </si>
   <si>
@@ -265,6 +274,15 @@
     <t>13:52:00 UTC</t>
   </si>
   <si>
+    <t>16:10:00 UTC</t>
+  </si>
+  <si>
+    <t>12:15:00 UTC</t>
+  </si>
+  <si>
+    <t>18:43:00 UTC</t>
+  </si>
+  <si>
     <t>GPA.3358-1016-7927-87380</t>
   </si>
   <si>
@@ -418,6 +436,15 @@
     <t>wp2T7taN7vXwuGSeb_P7hQ==</t>
   </si>
   <si>
+    <t>B0I50BbwEi2eCG_FNqXodQ==</t>
+  </si>
+  <si>
+    <t>_1qdKP7Kr3peK4W9FUqjsA==</t>
+  </si>
+  <si>
+    <t>cUZ8Id1TrqkwDjvZwgBKnw==</t>
+  </si>
+  <si>
     <t>Play Store</t>
   </si>
   <si>
@@ -580,6 +607,15 @@
     <t>KA 562130 India</t>
   </si>
   <si>
+    <t>FL 34208, United States</t>
+  </si>
+  <si>
+    <t>San Francisco, CA 94104-5401 United States</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
     <t>United Kingdom</t>
   </si>
   <si>
@@ -592,9 +628,6 @@
     <t>South Korea</t>
   </si>
   <si>
-    <t>Germany</t>
-  </si>
-  <si>
     <t>Pakistan</t>
   </si>
   <si>
@@ -730,6 +763,9 @@
     <t>USD 2.34</t>
   </si>
   <si>
+    <t>USD 0.99</t>
+  </si>
+  <si>
     <t>$0.99</t>
   </si>
   <si>
@@ -905,6 +941,9 @@
   </si>
   <si>
     <t>USD 1.59</t>
+  </si>
+  <si>
+    <t>USD 0.79</t>
   </si>
   <si>
     <t>App Sales</t>
@@ -1278,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -1333,31 +1372,31 @@
         <v>45934</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F2" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G2" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H2" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I2" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="J2" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="L2" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1368,31 +1407,31 @@
         <v>45935</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="H3" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="I3" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="J3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="L3" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1403,31 +1442,31 @@
         <v>45935</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F4" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G4" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="H4" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I4" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="J4" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="L4" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1438,31 +1477,31 @@
         <v>45936</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G5" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="H5" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="I5" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="J5" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="L5" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1473,31 +1512,31 @@
         <v>45938</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F6" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G6" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="H6" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="I6" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="J6" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="L6" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1508,31 +1547,31 @@
         <v>45940</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E7" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G7" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H7" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="I7" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="J7" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="L7" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1543,31 +1582,31 @@
         <v>45941</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F8" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G8" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="H8" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I8" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="J8" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="L8" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1578,31 +1617,31 @@
         <v>45942</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G9" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="H9" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="I9" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="J9" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="L9" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1613,31 +1652,31 @@
         <v>45942</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F10" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G10" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="H10" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I10" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="J10" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="L10" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1648,31 +1687,31 @@
         <v>45942</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E11" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F11" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G11" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="H11" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="I11" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="J11" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="L11" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1683,34 +1722,34 @@
         <v>45942</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F12" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G12" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H12" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="I12" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="J12" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K12" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="L12" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1721,31 +1760,31 @@
         <v>45945</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F13" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G13" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="H13" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="I13" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="J13" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="L13" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1756,31 +1795,31 @@
         <v>45945</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E14" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F14" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G14" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="H14" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="I14" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="J14" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="L14" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1791,31 +1830,31 @@
         <v>45946</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E15" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F15" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G15" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H15" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="I15" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="J15" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="L15" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -1826,34 +1865,34 @@
         <v>45946</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F16" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G16" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H16" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I16" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="J16" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K16" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="L16" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1864,34 +1903,34 @@
         <v>45947</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D17" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F17" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G17" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H17" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I17" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="J17" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1902,31 +1941,31 @@
         <v>45949</v>
       </c>
       <c r="C18" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E18" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F18" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G18" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H18" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I18" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="J18" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="L18" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1937,31 +1976,31 @@
         <v>45950</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D19" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F19" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G19" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="H19" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I19" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="J19" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="L19" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1972,31 +2011,31 @@
         <v>45951</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F20" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G20" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="H20" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I20" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="J20" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="L20" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2007,31 +2046,31 @@
         <v>45953</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D21" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F21" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G21" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="H21" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="I21" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="J21" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="L21" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2042,31 +2081,31 @@
         <v>45953</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D22" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E22" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F22" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G22" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="H22" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I22" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="J22" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="L22" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2077,31 +2116,31 @@
         <v>45954</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F23" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G23" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="H23" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I23" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="J23" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="L23" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2112,31 +2151,31 @@
         <v>45955</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E24" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F24" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G24" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="H24" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I24" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="J24" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="L24" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2147,34 +2186,34 @@
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D25" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E25" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F25" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G25" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="H25" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="I25" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="J25" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2185,34 +2224,34 @@
         <v>45956</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D26" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F26" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G26" t="s">
+        <v>173</v>
+      </c>
+      <c r="H26" t="s">
         <v>164</v>
       </c>
-      <c r="H26" t="s">
-        <v>155</v>
-      </c>
       <c r="I26" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="J26" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="K26" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="L26" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2223,34 +2262,34 @@
         <v>45957</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F27" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G27" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H27" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I27" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="J27" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K27">
         <v>0</v>
       </c>
       <c r="L27" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -2261,31 +2300,31 @@
         <v>45957</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E28" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F28" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G28" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="H28" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="I28" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="J28" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="L28" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2296,31 +2335,31 @@
         <v>45957</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E29" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F29" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G29" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="I29" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="J29" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="L29" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2331,34 +2370,34 @@
         <v>45957</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E30" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F30" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G30" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H30" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I30" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="J30" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="K30">
         <v>0</v>
       </c>
       <c r="L30" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -2369,34 +2408,34 @@
         <v>15</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D31" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E31" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F31" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G31" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="H31" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I31" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="J31" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="K31" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="L31" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -2407,34 +2446,34 @@
         <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E32" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F32" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G32" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H32" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="I32" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="J32" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="K32" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="L32" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -2445,34 +2484,34 @@
         <v>17</v>
       </c>
       <c r="C33" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E33" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F33" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G33" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="H33" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="I33" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="J33" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="K33" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="L33" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -2483,34 +2522,34 @@
         <v>18</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D34" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F34" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G34" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="H34" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="I34" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="J34" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="K34" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="L34" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -2521,34 +2560,34 @@
         <v>19</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F35" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G35" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="H35" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I35" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="J35" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="K35" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="L35" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -2559,34 +2598,34 @@
         <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E36" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F36" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G36" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="H36" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I36" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="J36" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="K36" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="L36" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -2597,34 +2636,34 @@
         <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F37" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G37" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="H37" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I37" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="J37" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="K37" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="L37" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -2635,34 +2674,34 @@
         <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E38" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="F38" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="G38" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="H38" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I38" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="J38" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="K38" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="L38" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -2673,34 +2712,34 @@
         <v>22</v>
       </c>
       <c r="C39" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G39" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="H39" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="I39" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="J39" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="K39" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="L39" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -2711,37 +2750,37 @@
         <v>23</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="E40" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G40" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H40" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="I40" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="J40" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="K40" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="L40" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="M40" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -2752,40 +2791,40 @@
         <v>23</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D41" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E41" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G41" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="H41" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I41" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="J41" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="K41" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="L41" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="M41" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="N41" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -2796,37 +2835,37 @@
         <v>23</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D42" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E42" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="F42" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="G42" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="H42" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I42" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="J42" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="K42" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="L42" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="M42" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -2837,37 +2876,37 @@
         <v>24</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D43" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E43" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F43" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G43" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="H43" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="I43" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="J43" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="K43" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="L43" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="M43" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -2878,37 +2917,37 @@
         <v>25</v>
       </c>
       <c r="C44" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D44" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E44" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F44" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G44" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="H44" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I44" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="J44" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="K44" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="L44" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="M44" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -2919,40 +2958,40 @@
         <v>26</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E45" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F45" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G45" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="H45" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="I45" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="J45" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="K45" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="L45" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="M45" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="N45" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -2963,37 +3002,37 @@
         <v>27</v>
       </c>
       <c r="C46" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D46" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E46" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F46" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G46" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="H46" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="I46" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="J46" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="K46" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="L46" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="M46" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -3004,37 +3043,37 @@
         <v>27</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D47" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E47" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="F47" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="G47" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="H47" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I47" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="J47" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="K47" t="s">
+        <v>256</v>
+      </c>
+      <c r="L47" t="s">
         <v>244</v>
       </c>
-      <c r="L47" t="s">
-        <v>233</v>
-      </c>
       <c r="M47" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -3045,37 +3084,37 @@
         <v>28</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D48" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="E48" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F48" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G48" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="H48" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="I48" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="J48" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="K48" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="L48" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="M48" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -3086,40 +3125,40 @@
         <v>29</v>
       </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D49" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E49" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F49" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G49" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="H49" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I49" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="J49" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="K49" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="L49" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="M49" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="N49" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -3130,37 +3169,37 @@
         <v>29</v>
       </c>
       <c r="C50" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D50" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E50" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F50" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="G50" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="H50" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="I50" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="J50" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="K50" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="L50" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="M50" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -3171,37 +3210,37 @@
         <v>30</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D51" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="E51" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F51" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="G51" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="H51" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="I51" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="J51" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="K51" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="L51" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="M51" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -3212,37 +3251,160 @@
         <v>31</v>
       </c>
       <c r="C52" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D52" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E52" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F52" t="s">
+        <v>149</v>
+      </c>
+      <c r="G52" t="s">
+        <v>196</v>
+      </c>
+      <c r="H52" t="s">
+        <v>183</v>
+      </c>
+      <c r="I52" t="s">
+        <v>248</v>
+      </c>
+      <c r="J52" t="s">
+        <v>216</v>
+      </c>
+      <c r="K52" t="s">
+        <v>271</v>
+      </c>
+      <c r="L52" t="s">
+        <v>308</v>
+      </c>
+      <c r="M52" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>32</v>
+      </c>
+      <c r="C53" t="s">
+        <v>86</v>
+      </c>
+      <c r="D53" t="s">
         <v>140</v>
       </c>
-      <c r="G52" t="s">
-        <v>187</v>
-      </c>
-      <c r="H52" t="s">
-        <v>174</v>
-      </c>
-      <c r="I52" t="s">
-        <v>237</v>
-      </c>
-      <c r="J52" t="s">
-        <v>205</v>
-      </c>
-      <c r="K52" t="s">
-        <v>259</v>
-      </c>
-      <c r="L52" t="s">
-        <v>296</v>
-      </c>
-      <c r="M52" t="s">
-        <v>299</v>
+      <c r="E53" t="s">
+        <v>144</v>
+      </c>
+      <c r="F53" t="s">
+        <v>146</v>
+      </c>
+      <c r="G53" t="s">
+        <v>197</v>
+      </c>
+      <c r="H53" t="s">
+        <v>164</v>
+      </c>
+      <c r="I53" t="s">
+        <v>249</v>
+      </c>
+      <c r="J53" t="s">
+        <v>249</v>
+      </c>
+      <c r="K53" t="s">
+        <v>269</v>
+      </c>
+      <c r="L53" t="s">
+        <v>309</v>
+      </c>
+      <c r="M53" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54" t="s">
+        <v>87</v>
+      </c>
+      <c r="D54" t="s">
+        <v>141</v>
+      </c>
+      <c r="E54" t="s">
+        <v>144</v>
+      </c>
+      <c r="F54" t="s">
+        <v>146</v>
+      </c>
+      <c r="G54" t="s">
+        <v>198</v>
+      </c>
+      <c r="H54" t="s">
+        <v>164</v>
+      </c>
+      <c r="I54" t="s">
+        <v>246</v>
+      </c>
+      <c r="J54" t="s">
+        <v>246</v>
+      </c>
+      <c r="K54" t="s">
+        <v>269</v>
+      </c>
+      <c r="L54" t="s">
+        <v>307</v>
+      </c>
+      <c r="M54" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" t="s">
+        <v>142</v>
+      </c>
+      <c r="E55" t="s">
+        <v>144</v>
+      </c>
+      <c r="F55" t="s">
+        <v>149</v>
+      </c>
+      <c r="G55" t="s">
+        <v>199</v>
+      </c>
+      <c r="H55" t="s">
+        <v>199</v>
+      </c>
+      <c r="I55" t="s">
+        <v>246</v>
+      </c>
+      <c r="J55" t="s">
+        <v>246</v>
+      </c>
+      <c r="K55" t="s">
+        <v>269</v>
+      </c>
+      <c r="L55" t="s">
+        <v>307</v>
+      </c>
+      <c r="M55" t="s">
+        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>